<commit_message>
Add input validation and refactor core function
</commit_message>
<xml_diff>
--- a/journal.xlsx
+++ b/journal.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="63">
   <si>
     <t>Last name</t>
     <phoneticPr fontId="1"/>
@@ -209,6 +209,86 @@
   </si>
   <si>
     <t>2026-09-02 15:31:50</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Taisia</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2026-09-04 13:50:41</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>NICIPURENCO</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ALEXANDRA</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2026-09-15 09:43:44</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>MAria</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2026-09-15 09:45:26</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2026-09-15 09:50:01</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Nicipurenco Serghei</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Serghei</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2026-09-15 09:50:13</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Ahramenco</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Denis</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2026-09-15 09:51:02</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>$$$$</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2026-09-15 09:54:13</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2026-09-15 09:58:16</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Ничипуренко</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Таисия</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2026-09-15 09:58:24</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -558,7 +638,7 @@
 
 <file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0">
@@ -785,6 +865,132 @@
         <v>42</v>
       </c>
     </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0">
+      <c r="A17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17">
+        <v>5</v>
+      </c>
+      <c r="D17" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0">
+      <c r="A18" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18">
+        <v>11</v>
+      </c>
+      <c r="D18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0">
+      <c r="A19" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" t="s">
+        <v>48</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0">
+      <c r="A20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B20" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20">
+        <v>19</v>
+      </c>
+      <c r="D20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0">
+      <c r="A21" t="s">
+        <v>51</v>
+      </c>
+      <c r="B21" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21">
+        <v>15</v>
+      </c>
+      <c r="D21" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0">
+      <c r="A22" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22">
+        <v>5</v>
+      </c>
+      <c r="D22" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0">
+      <c r="A23" t="s">
+        <v>57</v>
+      </c>
+      <c r="B23">
+        <v>88282</v>
+      </c>
+      <c r="C23">
+        <v>2</v>
+      </c>
+      <c r="D23" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0">
+      <c r="A24" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24">
+        <v>19</v>
+      </c>
+      <c r="D24" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0">
+      <c r="A25" t="s">
+        <v>60</v>
+      </c>
+      <c r="B25" t="s">
+        <v>61</v>
+      </c>
+      <c r="C25">
+        <v>20</v>
+      </c>
+      <c r="D25" t="s">
+        <v>62</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>